<commit_message>
Give the demo workbook enough eGFR patients for a cohort model
Imported eGFR covered five of 14 demo patients, below the ten-patient model
minimum, so the headline cohort model path ended disabled. A reproducible
script adds lab-style CKD-EPI 2021 eGFR rows, computed from the same-day
creatinine, for the six patients with creatinine, sex and age (plus two rows
for patient 3). Golden fixtures use their own workbook copies and are unchanged.
The e2e availability test now checks that the demo fits by default and keeps
the unavailable explanation on a small synthetic sample.
</commit_message>
<xml_diff>
--- a/public/test_labs.xlsx
+++ b/public/test_labs.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H217"/>
+  <dimension ref="A1:H285"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5959,9 +5959,1777 @@
         <v>49</v>
       </c>
     </row>
+    <row r="218">
+      <c r="A218">
+        <v>3</v>
+      </c>
+      <c r="B218" s="1">
+        <v>44562.041666666664</v>
+      </c>
+      <c r="C218" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D218" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E218" t="str">
+        <v>74,1</v>
+      </c>
+      <c r="F218" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G218" t="str">
+        <v>w</v>
+      </c>
+      <c r="H218">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219">
+        <v>3</v>
+      </c>
+      <c r="B219" s="1">
+        <v>45292.041666666664</v>
+      </c>
+      <c r="C219" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D219" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E219" t="str">
+        <v>43,1</v>
+      </c>
+      <c r="F219" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G219" t="str">
+        <v>w</v>
+      </c>
+      <c r="H219">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220">
+        <v>4</v>
+      </c>
+      <c r="B220" s="1">
+        <v>44562.041666666664</v>
+      </c>
+      <c r="C220" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D220" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E220" t="str">
+        <v>91,7</v>
+      </c>
+      <c r="F220" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G220" t="str">
+        <v>m</v>
+      </c>
+      <c r="H220">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221">
+        <v>4</v>
+      </c>
+      <c r="B221" s="1">
+        <v>44652.083333333336</v>
+      </c>
+      <c r="C221" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D221" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E221" t="str">
+        <v>86,5</v>
+      </c>
+      <c r="F221" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G221" t="str">
+        <v>m</v>
+      </c>
+      <c r="H221">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222">
+        <v>4</v>
+      </c>
+      <c r="B222" s="1">
+        <v>44742.083333333336</v>
+      </c>
+      <c r="C222" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D222" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E222" t="str">
+        <v>81,8</v>
+      </c>
+      <c r="F222" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G222" t="str">
+        <v>m</v>
+      </c>
+      <c r="H222">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223">
+        <v>4</v>
+      </c>
+      <c r="B223" s="1">
+        <v>44832.083333333336</v>
+      </c>
+      <c r="C223" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D223" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E223" t="str">
+        <v>79,5</v>
+      </c>
+      <c r="F223" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G223" t="str">
+        <v>m</v>
+      </c>
+      <c r="H223">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224">
+        <v>4</v>
+      </c>
+      <c r="B224" s="1">
+        <v>44922.041666666664</v>
+      </c>
+      <c r="C224" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D224" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E224" t="str">
+        <v>73,2</v>
+      </c>
+      <c r="F224" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G224" t="str">
+        <v>m</v>
+      </c>
+      <c r="H224">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225">
+        <v>4</v>
+      </c>
+      <c r="B225" s="1">
+        <v>45012.083333333336</v>
+      </c>
+      <c r="C225" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D225" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E225" t="str">
+        <v>69,7</v>
+      </c>
+      <c r="F225" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G225" t="str">
+        <v>m</v>
+      </c>
+      <c r="H225">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226">
+        <v>4</v>
+      </c>
+      <c r="B226" s="1">
+        <v>45102.083333333336</v>
+      </c>
+      <c r="C226" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D226" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E226" t="str">
+        <v>66,5</v>
+      </c>
+      <c r="F226" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G226" t="str">
+        <v>m</v>
+      </c>
+      <c r="H226">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227">
+        <v>4</v>
+      </c>
+      <c r="B227" s="1">
+        <v>45192.083333333336</v>
+      </c>
+      <c r="C227" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D227" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E227" t="str">
+        <v>63,2</v>
+      </c>
+      <c r="F227" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G227" t="str">
+        <v>m</v>
+      </c>
+      <c r="H227">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228">
+        <v>6</v>
+      </c>
+      <c r="B228" s="1">
+        <v>44571.041666666664</v>
+      </c>
+      <c r="C228" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D228" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E228" t="str">
+        <v>65,5</v>
+      </c>
+      <c r="F228" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G228" t="str">
+        <v>m</v>
+      </c>
+      <c r="H228">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229">
+        <v>6</v>
+      </c>
+      <c r="B229" s="1">
+        <v>44661.083333333336</v>
+      </c>
+      <c r="C229" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D229" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E229" t="str">
+        <v>62,3</v>
+      </c>
+      <c r="F229" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G229" t="str">
+        <v>m</v>
+      </c>
+      <c r="H229">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230">
+        <v>6</v>
+      </c>
+      <c r="B230" s="1">
+        <v>44752.083333333336</v>
+      </c>
+      <c r="C230" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D230" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E230" t="str">
+        <v>59,5</v>
+      </c>
+      <c r="F230" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G230" t="str">
+        <v>m</v>
+      </c>
+      <c r="H230">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231">
+        <v>6</v>
+      </c>
+      <c r="B231" s="1">
+        <v>44809.083333333336</v>
+      </c>
+      <c r="C231" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D231" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E231" t="str">
+        <v>59,1</v>
+      </c>
+      <c r="F231" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G231" t="str">
+        <v>m</v>
+      </c>
+      <c r="H231">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232">
+        <v>6</v>
+      </c>
+      <c r="B232" s="1">
+        <v>44812.083333333336</v>
+      </c>
+      <c r="C232" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D232" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E232" t="str">
+        <v>22,6</v>
+      </c>
+      <c r="F232" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G232" t="str">
+        <v>m</v>
+      </c>
+      <c r="H232">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233">
+        <v>6</v>
+      </c>
+      <c r="B233" s="1">
+        <v>44820.083333333336</v>
+      </c>
+      <c r="C233" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D233" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E233" t="str">
+        <v>35,2</v>
+      </c>
+      <c r="F233" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G233" t="str">
+        <v>m</v>
+      </c>
+      <c r="H233">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234">
+        <v>6</v>
+      </c>
+      <c r="B234" s="1">
+        <v>44832.083333333336</v>
+      </c>
+      <c r="C234" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D234" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E234" t="str">
+        <v>49,8</v>
+      </c>
+      <c r="F234" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G234" t="str">
+        <v>m</v>
+      </c>
+      <c r="H234">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235">
+        <v>6</v>
+      </c>
+      <c r="B235" s="1">
+        <v>44905.041666666664</v>
+      </c>
+      <c r="C235" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D235" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E235" t="str">
+        <v>56,5</v>
+      </c>
+      <c r="F235" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G235" t="str">
+        <v>m</v>
+      </c>
+      <c r="H235">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236">
+        <v>6</v>
+      </c>
+      <c r="B236" s="1">
+        <v>44995.041666666664</v>
+      </c>
+      <c r="C236" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D236" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E236" t="str">
+        <v>54,1</v>
+      </c>
+      <c r="F236" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G236" t="str">
+        <v>m</v>
+      </c>
+      <c r="H236">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237">
+        <v>6</v>
+      </c>
+      <c r="B237" s="1">
+        <v>45087.083333333336</v>
+      </c>
+      <c r="C237" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D237" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E237" t="str">
+        <v>51,8</v>
+      </c>
+      <c r="F237" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G237" t="str">
+        <v>m</v>
+      </c>
+      <c r="H237">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238">
+        <v>6</v>
+      </c>
+      <c r="B238" s="1">
+        <v>45179.083333333336</v>
+      </c>
+      <c r="C238" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D238" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E238" t="str">
+        <v>49,5</v>
+      </c>
+      <c r="F238" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G238" t="str">
+        <v>m</v>
+      </c>
+      <c r="H238">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239">
+        <v>7</v>
+      </c>
+      <c r="B239" s="1">
+        <v>44197.041666666664</v>
+      </c>
+      <c r="C239" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D239" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E239" t="str">
+        <v>80,0</v>
+      </c>
+      <c r="F239" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G239" t="str">
+        <v>m</v>
+      </c>
+      <c r="H239">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240">
+        <v>7</v>
+      </c>
+      <c r="B240" s="1">
+        <v>44256.041666666664</v>
+      </c>
+      <c r="C240" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D240" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E240" t="str">
+        <v>75,4</v>
+      </c>
+      <c r="F240" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G240" t="str">
+        <v>m</v>
+      </c>
+      <c r="H240">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241">
+        <v>7</v>
+      </c>
+      <c r="B241" s="1">
+        <v>44348.083333333336</v>
+      </c>
+      <c r="C241" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D241" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E241" t="str">
+        <v>71,3</v>
+      </c>
+      <c r="F241" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G241" t="str">
+        <v>m</v>
+      </c>
+      <c r="H241">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242">
+        <v>7</v>
+      </c>
+      <c r="B242" s="1">
+        <v>44350.083333333336</v>
+      </c>
+      <c r="C242" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D242" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E242" t="str">
+        <v>47,3</v>
+      </c>
+      <c r="F242" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G242" t="str">
+        <v>m</v>
+      </c>
+      <c r="H242">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243">
+        <v>7</v>
+      </c>
+      <c r="B243" s="1">
+        <v>44359.083333333336</v>
+      </c>
+      <c r="C243" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D243" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E243" t="str">
+        <v>64,3</v>
+      </c>
+      <c r="F243" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G243" t="str">
+        <v>m</v>
+      </c>
+      <c r="H243">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244">
+        <v>7</v>
+      </c>
+      <c r="B244" s="1">
+        <v>44440.083333333336</v>
+      </c>
+      <c r="C244" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D244" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E244" t="str">
+        <v>70,9</v>
+      </c>
+      <c r="F244" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G244" t="str">
+        <v>m</v>
+      </c>
+      <c r="H244">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245">
+        <v>7</v>
+      </c>
+      <c r="B245" s="1">
+        <v>44562.041666666664</v>
+      </c>
+      <c r="C245" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D245" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E245" t="str">
+        <v>67,2</v>
+      </c>
+      <c r="F245" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G245" t="str">
+        <v>m</v>
+      </c>
+      <c r="H245">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246">
+        <v>7</v>
+      </c>
+      <c r="B246" s="1">
+        <v>44565.041666666664</v>
+      </c>
+      <c r="C246" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D246" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E246" t="str">
+        <v>28,5</v>
+      </c>
+      <c r="F246" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G246" t="str">
+        <v>m</v>
+      </c>
+      <c r="H246">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247">
+        <v>7</v>
+      </c>
+      <c r="B247" s="1">
+        <v>44581.041666666664</v>
+      </c>
+      <c r="C247" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D247" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E247" t="str">
+        <v>55,4</v>
+      </c>
+      <c r="F247" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G247" t="str">
+        <v>m</v>
+      </c>
+      <c r="H247">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248">
+        <v>7</v>
+      </c>
+      <c r="B248" s="1">
+        <v>44713.083333333336</v>
+      </c>
+      <c r="C248" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D248" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E248" t="str">
+        <v>63,9</v>
+      </c>
+      <c r="F248" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G248" t="str">
+        <v>m</v>
+      </c>
+      <c r="H248">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249">
+        <v>7</v>
+      </c>
+      <c r="B249" s="1">
+        <v>44835.083333333336</v>
+      </c>
+      <c r="C249" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D249" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E249" t="str">
+        <v>60,4</v>
+      </c>
+      <c r="F249" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G249" t="str">
+        <v>m</v>
+      </c>
+      <c r="H249">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250">
+        <v>7</v>
+      </c>
+      <c r="B250" s="1">
+        <v>44837.083333333336</v>
+      </c>
+      <c r="C250" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D250" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E250" t="str">
+        <v>14,1</v>
+      </c>
+      <c r="F250" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G250" t="str">
+        <v>m</v>
+      </c>
+      <c r="H250">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251">
+        <v>7</v>
+      </c>
+      <c r="B251" s="1">
+        <v>44852.083333333336</v>
+      </c>
+      <c r="C251" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D251" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E251" t="str">
+        <v>34,4</v>
+      </c>
+      <c r="F251" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G251" t="str">
+        <v>m</v>
+      </c>
+      <c r="H251">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252">
+        <v>7</v>
+      </c>
+      <c r="B252" s="1">
+        <v>44927.041666666664</v>
+      </c>
+      <c r="C252" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D252" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E252" t="str">
+        <v>55,1</v>
+      </c>
+      <c r="F252" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G252" t="str">
+        <v>m</v>
+      </c>
+      <c r="H252">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253">
+        <v>7</v>
+      </c>
+      <c r="B253" s="1">
+        <v>45078.083333333336</v>
+      </c>
+      <c r="C253" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D253" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E253" t="str">
+        <v>52,7</v>
+      </c>
+      <c r="F253" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G253" t="str">
+        <v>m</v>
+      </c>
+      <c r="H253">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254">
+        <v>8</v>
+      </c>
+      <c r="B254" s="1">
+        <v>43862.041666666664</v>
+      </c>
+      <c r="C254" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D254" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E254" t="str">
+        <v>69,9</v>
+      </c>
+      <c r="F254" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G254" t="str">
+        <v>w</v>
+      </c>
+      <c r="H254">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255">
+        <v>8</v>
+      </c>
+      <c r="B255" s="1">
+        <v>44044.083333333336</v>
+      </c>
+      <c r="C255" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D255" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E255" t="str">
+        <v>68,2</v>
+      </c>
+      <c r="F255" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G255" t="str">
+        <v>w</v>
+      </c>
+      <c r="H255">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256">
+        <v>8</v>
+      </c>
+      <c r="B256" s="1">
+        <v>44228.041666666664</v>
+      </c>
+      <c r="C256" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D256" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E256" t="str">
+        <v>68,6</v>
+      </c>
+      <c r="F256" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G256" t="str">
+        <v>w</v>
+      </c>
+      <c r="H256">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257">
+        <v>8</v>
+      </c>
+      <c r="B257" s="1">
+        <v>44409.083333333336</v>
+      </c>
+      <c r="C257" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D257" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E257" t="str">
+        <v>66,9</v>
+      </c>
+      <c r="F257" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G257" t="str">
+        <v>w</v>
+      </c>
+      <c r="H257">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258">
+        <v>8</v>
+      </c>
+      <c r="B258" s="1">
+        <v>44593.041666666664</v>
+      </c>
+      <c r="C258" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D258" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E258" t="str">
+        <v>65,7</v>
+      </c>
+      <c r="F258" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G258" t="str">
+        <v>w</v>
+      </c>
+      <c r="H258">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259">
+        <v>8</v>
+      </c>
+      <c r="B259" s="1">
+        <v>44774.083333333336</v>
+      </c>
+      <c r="C259" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D259" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E259" t="str">
+        <v>67,3</v>
+      </c>
+      <c r="F259" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G259" t="str">
+        <v>w</v>
+      </c>
+      <c r="H259">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260">
+        <v>8</v>
+      </c>
+      <c r="B260" s="1">
+        <v>44958.041666666664</v>
+      </c>
+      <c r="C260" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D260" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E260" t="str">
+        <v>66,1</v>
+      </c>
+      <c r="F260" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G260" t="str">
+        <v>w</v>
+      </c>
+      <c r="H260">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261">
+        <v>8</v>
+      </c>
+      <c r="B261" s="1">
+        <v>45139.083333333336</v>
+      </c>
+      <c r="C261" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D261" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E261" t="str">
+        <v>64,5</v>
+      </c>
+      <c r="F261" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G261" t="str">
+        <v>w</v>
+      </c>
+      <c r="H261">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262">
+        <v>8</v>
+      </c>
+      <c r="B262" s="1">
+        <v>45323.041666666664</v>
+      </c>
+      <c r="C262" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D262" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E262" t="str">
+        <v>64,9</v>
+      </c>
+      <c r="F262" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G262" t="str">
+        <v>w</v>
+      </c>
+      <c r="H262">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263">
+        <v>8</v>
+      </c>
+      <c r="B263" s="1">
+        <v>45505.083333333336</v>
+      </c>
+      <c r="C263" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D263" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E263" t="str">
+        <v>63,4</v>
+      </c>
+      <c r="F263" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G263" t="str">
+        <v>w</v>
+      </c>
+      <c r="H263">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264">
+        <v>8</v>
+      </c>
+      <c r="B264" s="1">
+        <v>45689.041666666664</v>
+      </c>
+      <c r="C264" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D264" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E264" t="str">
+        <v>63,7</v>
+      </c>
+      <c r="F264" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G264" t="str">
+        <v>w</v>
+      </c>
+      <c r="H264">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265">
+        <v>8</v>
+      </c>
+      <c r="B265" s="1">
+        <v>45870.083333333336</v>
+      </c>
+      <c r="C265" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D265" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E265" t="str">
+        <v>62,2</v>
+      </c>
+      <c r="F265" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G265" t="str">
+        <v>w</v>
+      </c>
+      <c r="H265">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266">
+        <v>9</v>
+      </c>
+      <c r="B266" s="1">
+        <v>43497.041666666664</v>
+      </c>
+      <c r="C266" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D266" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E266" t="str">
+        <v>68,2</v>
+      </c>
+      <c r="F266" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G266" t="str">
+        <v>w</v>
+      </c>
+      <c r="H266">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267">
+        <v>9</v>
+      </c>
+      <c r="B267" s="1">
+        <v>43739.083333333336</v>
+      </c>
+      <c r="C267" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D267" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E267" t="str">
+        <v>61,4</v>
+      </c>
+      <c r="F267" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G267" t="str">
+        <v>w</v>
+      </c>
+      <c r="H267">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268">
+        <v>9</v>
+      </c>
+      <c r="B268" s="1">
+        <v>43983.083333333336</v>
+      </c>
+      <c r="C268" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D268" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E268" t="str">
+        <v>56,0</v>
+      </c>
+      <c r="F268" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G268" t="str">
+        <v>w</v>
+      </c>
+      <c r="H268">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269">
+        <v>9</v>
+      </c>
+      <c r="B269" s="1">
+        <v>44228.041666666664</v>
+      </c>
+      <c r="C269" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D269" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E269" t="str">
+        <v>50,0</v>
+      </c>
+      <c r="F269" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G269" t="str">
+        <v>w</v>
+      </c>
+      <c r="H269">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270">
+        <v>9</v>
+      </c>
+      <c r="B270" s="1">
+        <v>44470.083333333336</v>
+      </c>
+      <c r="C270" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D270" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E270" t="str">
+        <v>43,4</v>
+      </c>
+      <c r="F270" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G270" t="str">
+        <v>w</v>
+      </c>
+      <c r="H270">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271">
+        <v>9</v>
+      </c>
+      <c r="B271" s="1">
+        <v>44713.083333333336</v>
+      </c>
+      <c r="C271" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D271" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E271" t="str">
+        <v>37,9</v>
+      </c>
+      <c r="F271" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G271" t="str">
+        <v>w</v>
+      </c>
+      <c r="H271">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272">
+        <v>9</v>
+      </c>
+      <c r="B272" s="1">
+        <v>44958.041666666664</v>
+      </c>
+      <c r="C272" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D272" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E272" t="str">
+        <v>33,0</v>
+      </c>
+      <c r="F272" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G272" t="str">
+        <v>w</v>
+      </c>
+      <c r="H272">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273">
+        <v>9</v>
+      </c>
+      <c r="B273" s="1">
+        <v>45200.083333333336</v>
+      </c>
+      <c r="C273" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D273" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E273" t="str">
+        <v>29,2</v>
+      </c>
+      <c r="F273" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G273" t="str">
+        <v>w</v>
+      </c>
+      <c r="H273">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274">
+        <v>9</v>
+      </c>
+      <c r="B274" s="1">
+        <v>45444.083333333336</v>
+      </c>
+      <c r="C274" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D274" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E274" t="str">
+        <v>25,7</v>
+      </c>
+      <c r="F274" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G274" t="str">
+        <v>w</v>
+      </c>
+      <c r="H274">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275">
+        <v>9</v>
+      </c>
+      <c r="B275" s="1">
+        <v>45689.041666666664</v>
+      </c>
+      <c r="C275" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D275" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E275" t="str">
+        <v>22,6</v>
+      </c>
+      <c r="F275" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G275" t="str">
+        <v>w</v>
+      </c>
+      <c r="H275">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276">
+        <v>12</v>
+      </c>
+      <c r="B276" s="1">
+        <v>44197.041666666664</v>
+      </c>
+      <c r="C276" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D276" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E276" t="str">
+        <v>59,1</v>
+      </c>
+      <c r="F276" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G276" t="str">
+        <v>w</v>
+      </c>
+      <c r="H276">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277">
+        <v>12</v>
+      </c>
+      <c r="B277" s="1">
+        <v>44199.041666666664</v>
+      </c>
+      <c r="C277" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D277" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E277" t="str">
+        <v>39,5</v>
+      </c>
+      <c r="F277" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G277" t="str">
+        <v>w</v>
+      </c>
+      <c r="H277">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278">
+        <v>12</v>
+      </c>
+      <c r="B278" s="1">
+        <v>44216.041666666664</v>
+      </c>
+      <c r="C278" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D278" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E278" t="str">
+        <v>55,8</v>
+      </c>
+      <c r="F278" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G278" t="str">
+        <v>w</v>
+      </c>
+      <c r="H278">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279">
+        <v>12</v>
+      </c>
+      <c r="B279" s="1">
+        <v>44242.041666666664</v>
+      </c>
+      <c r="C279" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D279" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E279" t="str">
+        <v>59,1</v>
+      </c>
+      <c r="F279" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G279" t="str">
+        <v>w</v>
+      </c>
+      <c r="H279">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280">
+        <v>12</v>
+      </c>
+      <c r="B280" s="1">
+        <v>44244.041666666664</v>
+      </c>
+      <c r="C280" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D280" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E280" t="str">
+        <v>41,2</v>
+      </c>
+      <c r="F280" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G280" t="str">
+        <v>w</v>
+      </c>
+      <c r="H280">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281">
+        <v>12</v>
+      </c>
+      <c r="B281" s="1">
+        <v>44265.041666666664</v>
+      </c>
+      <c r="C281" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D281" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E281" t="str">
+        <v>55,8</v>
+      </c>
+      <c r="F281" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G281" t="str">
+        <v>w</v>
+      </c>
+      <c r="H281">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282">
+        <v>12</v>
+      </c>
+      <c r="B282" s="1">
+        <v>44287.083333333336</v>
+      </c>
+      <c r="C282" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D282" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E282" t="str">
+        <v>59,1</v>
+      </c>
+      <c r="F282" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G282" t="str">
+        <v>w</v>
+      </c>
+      <c r="H282">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283">
+        <v>12</v>
+      </c>
+      <c r="B283" s="1">
+        <v>44289.083333333336</v>
+      </c>
+      <c r="C283" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D283" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E283" t="str">
+        <v>25,0</v>
+      </c>
+      <c r="F283" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G283" t="str">
+        <v>w</v>
+      </c>
+      <c r="H283">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284">
+        <v>12</v>
+      </c>
+      <c r="B284" s="1">
+        <v>44306.083333333336</v>
+      </c>
+      <c r="C284" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D284" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E284" t="str">
+        <v>47,5</v>
+      </c>
+      <c r="F284" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G284" t="str">
+        <v>w</v>
+      </c>
+      <c r="H284">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285">
+        <v>12</v>
+      </c>
+      <c r="B285" s="1">
+        <v>44348.083333333336</v>
+      </c>
+      <c r="C285" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D285" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E285" t="str">
+        <v>53,9</v>
+      </c>
+      <c r="F285" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G285" t="str">
+        <v>w</v>
+      </c>
+      <c r="H285">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H217"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H285"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Address branch review: validated preselection, demo eGFR, formatting
- Preselection pre-check counts only exact measurements (a '>90' eGFR no
  longer counts) in one pass, and the chosen candidate must pass the real
  preparation and validation with the standard model, checked lazily.
- Method reference describes the new preselection rule; changelog wording
  follows it.
- Demo script treats any eGFR series as existing, so patient 3 no longer gets
  conflicting rows; workbook regenerated (282 rows, eGFR for 11 patients).
- Display numbers never read '-0'; detail values use the shared formatter,
  the coefficient table keeps fixed decimals.
- Singular count in chart export context, CSS artefact removed, trend
  heading aligned with the switch, dated smoke checklist entry.
</commit_message>
<xml_diff>
--- a/public/test_labs.xlsx
+++ b/public/test_labs.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H285"/>
+  <dimension ref="A1:H283"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5961,7 +5961,7 @@
     </row>
     <row r="218">
       <c r="A218">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B218" s="1">
         <v>44562.041666666664</v>
@@ -5973,24 +5973,24 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E218" t="str">
-        <v>74,1</v>
+        <v>91,7</v>
       </c>
       <c r="F218" t="str">
         <v>98979-8</v>
       </c>
       <c r="G218" t="str">
-        <v>w</v>
+        <v>m</v>
       </c>
       <c r="H218">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="219">
       <c r="A219">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B219" s="1">
-        <v>45292.041666666664</v>
+        <v>44652.083333333336</v>
       </c>
       <c r="C219" t="str">
         <v>eGFR</v>
@@ -5999,16 +5999,16 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E219" t="str">
-        <v>43,1</v>
+        <v>86,5</v>
       </c>
       <c r="F219" t="str">
         <v>98979-8</v>
       </c>
       <c r="G219" t="str">
-        <v>w</v>
+        <v>m</v>
       </c>
       <c r="H219">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="220">
@@ -6016,7 +6016,7 @@
         <v>4</v>
       </c>
       <c r="B220" s="1">
-        <v>44562.041666666664</v>
+        <v>44742.083333333336</v>
       </c>
       <c r="C220" t="str">
         <v>eGFR</v>
@@ -6025,7 +6025,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E220" t="str">
-        <v>91,7</v>
+        <v>81,8</v>
       </c>
       <c r="F220" t="str">
         <v>98979-8</v>
@@ -6042,7 +6042,7 @@
         <v>4</v>
       </c>
       <c r="B221" s="1">
-        <v>44652.083333333336</v>
+        <v>44832.083333333336</v>
       </c>
       <c r="C221" t="str">
         <v>eGFR</v>
@@ -6051,7 +6051,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E221" t="str">
-        <v>86,5</v>
+        <v>79,5</v>
       </c>
       <c r="F221" t="str">
         <v>98979-8</v>
@@ -6060,7 +6060,7 @@
         <v>m</v>
       </c>
       <c r="H221">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="222">
@@ -6068,7 +6068,7 @@
         <v>4</v>
       </c>
       <c r="B222" s="1">
-        <v>44742.083333333336</v>
+        <v>44922.041666666664</v>
       </c>
       <c r="C222" t="str">
         <v>eGFR</v>
@@ -6077,7 +6077,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E222" t="str">
-        <v>81,8</v>
+        <v>73,2</v>
       </c>
       <c r="F222" t="str">
         <v>98979-8</v>
@@ -6086,7 +6086,7 @@
         <v>m</v>
       </c>
       <c r="H222">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="223">
@@ -6094,7 +6094,7 @@
         <v>4</v>
       </c>
       <c r="B223" s="1">
-        <v>44832.083333333336</v>
+        <v>45012.083333333336</v>
       </c>
       <c r="C223" t="str">
         <v>eGFR</v>
@@ -6103,7 +6103,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E223" t="str">
-        <v>79,5</v>
+        <v>69,7</v>
       </c>
       <c r="F223" t="str">
         <v>98979-8</v>
@@ -6120,7 +6120,7 @@
         <v>4</v>
       </c>
       <c r="B224" s="1">
-        <v>44922.041666666664</v>
+        <v>45102.083333333336</v>
       </c>
       <c r="C224" t="str">
         <v>eGFR</v>
@@ -6129,7 +6129,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E224" t="str">
-        <v>73,2</v>
+        <v>66,5</v>
       </c>
       <c r="F224" t="str">
         <v>98979-8</v>
@@ -6146,7 +6146,7 @@
         <v>4</v>
       </c>
       <c r="B225" s="1">
-        <v>45012.083333333336</v>
+        <v>45192.083333333336</v>
       </c>
       <c r="C225" t="str">
         <v>eGFR</v>
@@ -6155,7 +6155,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E225" t="str">
-        <v>69,7</v>
+        <v>63,2</v>
       </c>
       <c r="F225" t="str">
         <v>98979-8</v>
@@ -6164,15 +6164,15 @@
         <v>m</v>
       </c>
       <c r="H225">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="226">
       <c r="A226">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B226" s="1">
-        <v>45102.083333333336</v>
+        <v>44571.041666666664</v>
       </c>
       <c r="C226" t="str">
         <v>eGFR</v>
@@ -6181,7 +6181,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E226" t="str">
-        <v>66,5</v>
+        <v>65,5</v>
       </c>
       <c r="F226" t="str">
         <v>98979-8</v>
@@ -6190,15 +6190,15 @@
         <v>m</v>
       </c>
       <c r="H226">
-        <v>51</v>
+        <v>69</v>
       </c>
     </row>
     <row r="227">
       <c r="A227">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B227" s="1">
-        <v>45192.083333333336</v>
+        <v>44661.083333333336</v>
       </c>
       <c r="C227" t="str">
         <v>eGFR</v>
@@ -6207,7 +6207,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E227" t="str">
-        <v>63,2</v>
+        <v>62,3</v>
       </c>
       <c r="F227" t="str">
         <v>98979-8</v>
@@ -6216,7 +6216,7 @@
         <v>m</v>
       </c>
       <c r="H227">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="228">
@@ -6224,7 +6224,7 @@
         <v>6</v>
       </c>
       <c r="B228" s="1">
-        <v>44571.041666666664</v>
+        <v>44752.083333333336</v>
       </c>
       <c r="C228" t="str">
         <v>eGFR</v>
@@ -6233,7 +6233,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E228" t="str">
-        <v>65,5</v>
+        <v>59,5</v>
       </c>
       <c r="F228" t="str">
         <v>98979-8</v>
@@ -6250,7 +6250,7 @@
         <v>6</v>
       </c>
       <c r="B229" s="1">
-        <v>44661.083333333336</v>
+        <v>44809.083333333336</v>
       </c>
       <c r="C229" t="str">
         <v>eGFR</v>
@@ -6259,7 +6259,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E229" t="str">
-        <v>62,3</v>
+        <v>59,1</v>
       </c>
       <c r="F229" t="str">
         <v>98979-8</v>
@@ -6268,7 +6268,7 @@
         <v>m</v>
       </c>
       <c r="H229">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="230">
@@ -6276,7 +6276,7 @@
         <v>6</v>
       </c>
       <c r="B230" s="1">
-        <v>44752.083333333336</v>
+        <v>44812.083333333336</v>
       </c>
       <c r="C230" t="str">
         <v>eGFR</v>
@@ -6285,7 +6285,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E230" t="str">
-        <v>59,5</v>
+        <v>22,6</v>
       </c>
       <c r="F230" t="str">
         <v>98979-8</v>
@@ -6294,7 +6294,7 @@
         <v>m</v>
       </c>
       <c r="H230">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="231">
@@ -6302,7 +6302,7 @@
         <v>6</v>
       </c>
       <c r="B231" s="1">
-        <v>44809.083333333336</v>
+        <v>44820.083333333336</v>
       </c>
       <c r="C231" t="str">
         <v>eGFR</v>
@@ -6311,7 +6311,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E231" t="str">
-        <v>59,1</v>
+        <v>35,2</v>
       </c>
       <c r="F231" t="str">
         <v>98979-8</v>
@@ -6328,7 +6328,7 @@
         <v>6</v>
       </c>
       <c r="B232" s="1">
-        <v>44812.083333333336</v>
+        <v>44832.083333333336</v>
       </c>
       <c r="C232" t="str">
         <v>eGFR</v>
@@ -6337,7 +6337,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E232" t="str">
-        <v>22,6</v>
+        <v>49,8</v>
       </c>
       <c r="F232" t="str">
         <v>98979-8</v>
@@ -6354,7 +6354,7 @@
         <v>6</v>
       </c>
       <c r="B233" s="1">
-        <v>44820.083333333336</v>
+        <v>44905.041666666664</v>
       </c>
       <c r="C233" t="str">
         <v>eGFR</v>
@@ -6363,7 +6363,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E233" t="str">
-        <v>35,2</v>
+        <v>56,5</v>
       </c>
       <c r="F233" t="str">
         <v>98979-8</v>
@@ -6380,7 +6380,7 @@
         <v>6</v>
       </c>
       <c r="B234" s="1">
-        <v>44832.083333333336</v>
+        <v>44995.041666666664</v>
       </c>
       <c r="C234" t="str">
         <v>eGFR</v>
@@ -6389,7 +6389,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E234" t="str">
-        <v>49,8</v>
+        <v>54,1</v>
       </c>
       <c r="F234" t="str">
         <v>98979-8</v>
@@ -6406,7 +6406,7 @@
         <v>6</v>
       </c>
       <c r="B235" s="1">
-        <v>44905.041666666664</v>
+        <v>45087.083333333336</v>
       </c>
       <c r="C235" t="str">
         <v>eGFR</v>
@@ -6415,7 +6415,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E235" t="str">
-        <v>56,5</v>
+        <v>51,8</v>
       </c>
       <c r="F235" t="str">
         <v>98979-8</v>
@@ -6432,7 +6432,7 @@
         <v>6</v>
       </c>
       <c r="B236" s="1">
-        <v>44995.041666666664</v>
+        <v>45179.083333333336</v>
       </c>
       <c r="C236" t="str">
         <v>eGFR</v>
@@ -6441,7 +6441,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E236" t="str">
-        <v>54,1</v>
+        <v>49,5</v>
       </c>
       <c r="F236" t="str">
         <v>98979-8</v>
@@ -6450,15 +6450,15 @@
         <v>m</v>
       </c>
       <c r="H236">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="237">
       <c r="A237">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B237" s="1">
-        <v>45087.083333333336</v>
+        <v>44197.041666666664</v>
       </c>
       <c r="C237" t="str">
         <v>eGFR</v>
@@ -6467,7 +6467,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E237" t="str">
-        <v>51,8</v>
+        <v>80,0</v>
       </c>
       <c r="F237" t="str">
         <v>98979-8</v>
@@ -6476,15 +6476,15 @@
         <v>m</v>
       </c>
       <c r="H237">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="238">
       <c r="A238">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B238" s="1">
-        <v>45179.083333333336</v>
+        <v>44256.041666666664</v>
       </c>
       <c r="C238" t="str">
         <v>eGFR</v>
@@ -6493,7 +6493,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E238" t="str">
-        <v>49,5</v>
+        <v>75,4</v>
       </c>
       <c r="F238" t="str">
         <v>98979-8</v>
@@ -6502,7 +6502,7 @@
         <v>m</v>
       </c>
       <c r="H238">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="239">
@@ -6510,7 +6510,7 @@
         <v>7</v>
       </c>
       <c r="B239" s="1">
-        <v>44197.041666666664</v>
+        <v>44348.083333333336</v>
       </c>
       <c r="C239" t="str">
         <v>eGFR</v>
@@ -6519,7 +6519,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E239" t="str">
-        <v>80,0</v>
+        <v>71,3</v>
       </c>
       <c r="F239" t="str">
         <v>98979-8</v>
@@ -6536,7 +6536,7 @@
         <v>7</v>
       </c>
       <c r="B240" s="1">
-        <v>44256.041666666664</v>
+        <v>44350.083333333336</v>
       </c>
       <c r="C240" t="str">
         <v>eGFR</v>
@@ -6545,7 +6545,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E240" t="str">
-        <v>75,4</v>
+        <v>47,3</v>
       </c>
       <c r="F240" t="str">
         <v>98979-8</v>
@@ -6562,7 +6562,7 @@
         <v>7</v>
       </c>
       <c r="B241" s="1">
-        <v>44348.083333333336</v>
+        <v>44359.083333333336</v>
       </c>
       <c r="C241" t="str">
         <v>eGFR</v>
@@ -6571,7 +6571,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E241" t="str">
-        <v>71,3</v>
+        <v>64,3</v>
       </c>
       <c r="F241" t="str">
         <v>98979-8</v>
@@ -6588,7 +6588,7 @@
         <v>7</v>
       </c>
       <c r="B242" s="1">
-        <v>44350.083333333336</v>
+        <v>44440.083333333336</v>
       </c>
       <c r="C242" t="str">
         <v>eGFR</v>
@@ -6597,7 +6597,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E242" t="str">
-        <v>47,3</v>
+        <v>70,9</v>
       </c>
       <c r="F242" t="str">
         <v>98979-8</v>
@@ -6606,7 +6606,7 @@
         <v>m</v>
       </c>
       <c r="H242">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="243">
@@ -6614,7 +6614,7 @@
         <v>7</v>
       </c>
       <c r="B243" s="1">
-        <v>44359.083333333336</v>
+        <v>44562.041666666664</v>
       </c>
       <c r="C243" t="str">
         <v>eGFR</v>
@@ -6623,7 +6623,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E243" t="str">
-        <v>64,3</v>
+        <v>67,2</v>
       </c>
       <c r="F243" t="str">
         <v>98979-8</v>
@@ -6632,7 +6632,7 @@
         <v>m</v>
       </c>
       <c r="H243">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="244">
@@ -6640,7 +6640,7 @@
         <v>7</v>
       </c>
       <c r="B244" s="1">
-        <v>44440.083333333336</v>
+        <v>44565.041666666664</v>
       </c>
       <c r="C244" t="str">
         <v>eGFR</v>
@@ -6649,7 +6649,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E244" t="str">
-        <v>70,9</v>
+        <v>28,5</v>
       </c>
       <c r="F244" t="str">
         <v>98979-8</v>
@@ -6666,7 +6666,7 @@
         <v>7</v>
       </c>
       <c r="B245" s="1">
-        <v>44562.041666666664</v>
+        <v>44581.041666666664</v>
       </c>
       <c r="C245" t="str">
         <v>eGFR</v>
@@ -6675,7 +6675,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E245" t="str">
-        <v>67,2</v>
+        <v>55,4</v>
       </c>
       <c r="F245" t="str">
         <v>98979-8</v>
@@ -6692,7 +6692,7 @@
         <v>7</v>
       </c>
       <c r="B246" s="1">
-        <v>44565.041666666664</v>
+        <v>44713.083333333336</v>
       </c>
       <c r="C246" t="str">
         <v>eGFR</v>
@@ -6701,7 +6701,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E246" t="str">
-        <v>28,5</v>
+        <v>63,9</v>
       </c>
       <c r="F246" t="str">
         <v>98979-8</v>
@@ -6718,7 +6718,7 @@
         <v>7</v>
       </c>
       <c r="B247" s="1">
-        <v>44581.041666666664</v>
+        <v>44835.083333333336</v>
       </c>
       <c r="C247" t="str">
         <v>eGFR</v>
@@ -6727,7 +6727,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E247" t="str">
-        <v>55,4</v>
+        <v>60,4</v>
       </c>
       <c r="F247" t="str">
         <v>98979-8</v>
@@ -6736,7 +6736,7 @@
         <v>m</v>
       </c>
       <c r="H247">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="248">
@@ -6744,7 +6744,7 @@
         <v>7</v>
       </c>
       <c r="B248" s="1">
-        <v>44713.083333333336</v>
+        <v>44837.083333333336</v>
       </c>
       <c r="C248" t="str">
         <v>eGFR</v>
@@ -6753,7 +6753,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E248" t="str">
-        <v>63,9</v>
+        <v>14,1</v>
       </c>
       <c r="F248" t="str">
         <v>98979-8</v>
@@ -6762,7 +6762,7 @@
         <v>m</v>
       </c>
       <c r="H248">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="249">
@@ -6770,7 +6770,7 @@
         <v>7</v>
       </c>
       <c r="B249" s="1">
-        <v>44835.083333333336</v>
+        <v>44852.083333333336</v>
       </c>
       <c r="C249" t="str">
         <v>eGFR</v>
@@ -6779,7 +6779,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E249" t="str">
-        <v>60,4</v>
+        <v>34,4</v>
       </c>
       <c r="F249" t="str">
         <v>98979-8</v>
@@ -6796,7 +6796,7 @@
         <v>7</v>
       </c>
       <c r="B250" s="1">
-        <v>44837.083333333336</v>
+        <v>44927.041666666664</v>
       </c>
       <c r="C250" t="str">
         <v>eGFR</v>
@@ -6805,7 +6805,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E250" t="str">
-        <v>14,1</v>
+        <v>55,1</v>
       </c>
       <c r="F250" t="str">
         <v>98979-8</v>
@@ -6822,7 +6822,7 @@
         <v>7</v>
       </c>
       <c r="B251" s="1">
-        <v>44852.083333333336</v>
+        <v>45078.083333333336</v>
       </c>
       <c r="C251" t="str">
         <v>eGFR</v>
@@ -6831,7 +6831,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E251" t="str">
-        <v>34,4</v>
+        <v>52,7</v>
       </c>
       <c r="F251" t="str">
         <v>98979-8</v>
@@ -6845,10 +6845,10 @@
     </row>
     <row r="252">
       <c r="A252">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B252" s="1">
-        <v>44927.041666666664</v>
+        <v>43862.041666666664</v>
       </c>
       <c r="C252" t="str">
         <v>eGFR</v>
@@ -6857,24 +6857,24 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E252" t="str">
-        <v>55,1</v>
+        <v>69,9</v>
       </c>
       <c r="F252" t="str">
         <v>98979-8</v>
       </c>
       <c r="G252" t="str">
-        <v>m</v>
+        <v>w</v>
       </c>
       <c r="H252">
-        <v>74</v>
+        <v>55</v>
       </c>
     </row>
     <row r="253">
       <c r="A253">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B253" s="1">
-        <v>45078.083333333336</v>
+        <v>44044.083333333336</v>
       </c>
       <c r="C253" t="str">
         <v>eGFR</v>
@@ -6883,16 +6883,16 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E253" t="str">
-        <v>52,7</v>
+        <v>68,2</v>
       </c>
       <c r="F253" t="str">
         <v>98979-8</v>
       </c>
       <c r="G253" t="str">
-        <v>m</v>
+        <v>w</v>
       </c>
       <c r="H253">
-        <v>74</v>
+        <v>55</v>
       </c>
     </row>
     <row r="254">
@@ -6900,7 +6900,7 @@
         <v>8</v>
       </c>
       <c r="B254" s="1">
-        <v>43862.041666666664</v>
+        <v>44228.041666666664</v>
       </c>
       <c r="C254" t="str">
         <v>eGFR</v>
@@ -6909,7 +6909,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E254" t="str">
-        <v>69,9</v>
+        <v>68,6</v>
       </c>
       <c r="F254" t="str">
         <v>98979-8</v>
@@ -6918,7 +6918,7 @@
         <v>w</v>
       </c>
       <c r="H254">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="255">
@@ -6926,7 +6926,7 @@
         <v>8</v>
       </c>
       <c r="B255" s="1">
-        <v>44044.083333333336</v>
+        <v>44409.083333333336</v>
       </c>
       <c r="C255" t="str">
         <v>eGFR</v>
@@ -6935,7 +6935,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E255" t="str">
-        <v>68,2</v>
+        <v>66,9</v>
       </c>
       <c r="F255" t="str">
         <v>98979-8</v>
@@ -6944,7 +6944,7 @@
         <v>w</v>
       </c>
       <c r="H255">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="256">
@@ -6952,7 +6952,7 @@
         <v>8</v>
       </c>
       <c r="B256" s="1">
-        <v>44228.041666666664</v>
+        <v>44593.041666666664</v>
       </c>
       <c r="C256" t="str">
         <v>eGFR</v>
@@ -6961,7 +6961,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E256" t="str">
-        <v>68,6</v>
+        <v>65,7</v>
       </c>
       <c r="F256" t="str">
         <v>98979-8</v>
@@ -6970,7 +6970,7 @@
         <v>w</v>
       </c>
       <c r="H256">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="257">
@@ -6978,7 +6978,7 @@
         <v>8</v>
       </c>
       <c r="B257" s="1">
-        <v>44409.083333333336</v>
+        <v>44774.083333333336</v>
       </c>
       <c r="C257" t="str">
         <v>eGFR</v>
@@ -6987,7 +6987,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E257" t="str">
-        <v>66,9</v>
+        <v>67,3</v>
       </c>
       <c r="F257" t="str">
         <v>98979-8</v>
@@ -6996,7 +6996,7 @@
         <v>w</v>
       </c>
       <c r="H257">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="258">
@@ -7004,7 +7004,7 @@
         <v>8</v>
       </c>
       <c r="B258" s="1">
-        <v>44593.041666666664</v>
+        <v>44958.041666666664</v>
       </c>
       <c r="C258" t="str">
         <v>eGFR</v>
@@ -7013,7 +7013,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E258" t="str">
-        <v>65,7</v>
+        <v>66,1</v>
       </c>
       <c r="F258" t="str">
         <v>98979-8</v>
@@ -7022,7 +7022,7 @@
         <v>w</v>
       </c>
       <c r="H258">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="259">
@@ -7030,7 +7030,7 @@
         <v>8</v>
       </c>
       <c r="B259" s="1">
-        <v>44774.083333333336</v>
+        <v>45139.083333333336</v>
       </c>
       <c r="C259" t="str">
         <v>eGFR</v>
@@ -7039,7 +7039,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E259" t="str">
-        <v>67,3</v>
+        <v>64,5</v>
       </c>
       <c r="F259" t="str">
         <v>98979-8</v>
@@ -7048,7 +7048,7 @@
         <v>w</v>
       </c>
       <c r="H259">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="260">
@@ -7056,7 +7056,7 @@
         <v>8</v>
       </c>
       <c r="B260" s="1">
-        <v>44958.041666666664</v>
+        <v>45323.041666666664</v>
       </c>
       <c r="C260" t="str">
         <v>eGFR</v>
@@ -7065,7 +7065,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E260" t="str">
-        <v>66,1</v>
+        <v>64,9</v>
       </c>
       <c r="F260" t="str">
         <v>98979-8</v>
@@ -7074,7 +7074,7 @@
         <v>w</v>
       </c>
       <c r="H260">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="261">
@@ -7082,7 +7082,7 @@
         <v>8</v>
       </c>
       <c r="B261" s="1">
-        <v>45139.083333333336</v>
+        <v>45505.083333333336</v>
       </c>
       <c r="C261" t="str">
         <v>eGFR</v>
@@ -7091,7 +7091,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E261" t="str">
-        <v>64,5</v>
+        <v>63,4</v>
       </c>
       <c r="F261" t="str">
         <v>98979-8</v>
@@ -7100,7 +7100,7 @@
         <v>w</v>
       </c>
       <c r="H261">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="262">
@@ -7108,7 +7108,7 @@
         <v>8</v>
       </c>
       <c r="B262" s="1">
-        <v>45323.041666666664</v>
+        <v>45689.041666666664</v>
       </c>
       <c r="C262" t="str">
         <v>eGFR</v>
@@ -7117,7 +7117,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E262" t="str">
-        <v>64,9</v>
+        <v>63,7</v>
       </c>
       <c r="F262" t="str">
         <v>98979-8</v>
@@ -7126,7 +7126,7 @@
         <v>w</v>
       </c>
       <c r="H262">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="263">
@@ -7134,7 +7134,7 @@
         <v>8</v>
       </c>
       <c r="B263" s="1">
-        <v>45505.083333333336</v>
+        <v>45870.083333333336</v>
       </c>
       <c r="C263" t="str">
         <v>eGFR</v>
@@ -7143,7 +7143,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E263" t="str">
-        <v>63,4</v>
+        <v>62,2</v>
       </c>
       <c r="F263" t="str">
         <v>98979-8</v>
@@ -7152,15 +7152,15 @@
         <v>w</v>
       </c>
       <c r="H263">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="264">
       <c r="A264">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B264" s="1">
-        <v>45689.041666666664</v>
+        <v>43497.041666666664</v>
       </c>
       <c r="C264" t="str">
         <v>eGFR</v>
@@ -7169,7 +7169,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E264" t="str">
-        <v>63,7</v>
+        <v>68,2</v>
       </c>
       <c r="F264" t="str">
         <v>98979-8</v>
@@ -7178,15 +7178,15 @@
         <v>w</v>
       </c>
       <c r="H264">
-        <v>60</v>
+        <v>67</v>
       </c>
     </row>
     <row r="265">
       <c r="A265">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B265" s="1">
-        <v>45870.083333333336</v>
+        <v>43739.083333333336</v>
       </c>
       <c r="C265" t="str">
         <v>eGFR</v>
@@ -7195,7 +7195,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E265" t="str">
-        <v>62,2</v>
+        <v>61,4</v>
       </c>
       <c r="F265" t="str">
         <v>98979-8</v>
@@ -7204,7 +7204,7 @@
         <v>w</v>
       </c>
       <c r="H265">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="266">
@@ -7212,7 +7212,7 @@
         <v>9</v>
       </c>
       <c r="B266" s="1">
-        <v>43497.041666666664</v>
+        <v>43983.083333333336</v>
       </c>
       <c r="C266" t="str">
         <v>eGFR</v>
@@ -7221,7 +7221,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E266" t="str">
-        <v>68,2</v>
+        <v>56,0</v>
       </c>
       <c r="F266" t="str">
         <v>98979-8</v>
@@ -7230,7 +7230,7 @@
         <v>w</v>
       </c>
       <c r="H266">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="267">
@@ -7238,7 +7238,7 @@
         <v>9</v>
       </c>
       <c r="B267" s="1">
-        <v>43739.083333333336</v>
+        <v>44228.041666666664</v>
       </c>
       <c r="C267" t="str">
         <v>eGFR</v>
@@ -7247,7 +7247,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E267" t="str">
-        <v>61,4</v>
+        <v>50,0</v>
       </c>
       <c r="F267" t="str">
         <v>98979-8</v>
@@ -7256,7 +7256,7 @@
         <v>w</v>
       </c>
       <c r="H267">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="268">
@@ -7264,7 +7264,7 @@
         <v>9</v>
       </c>
       <c r="B268" s="1">
-        <v>43983.083333333336</v>
+        <v>44470.083333333336</v>
       </c>
       <c r="C268" t="str">
         <v>eGFR</v>
@@ -7273,7 +7273,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E268" t="str">
-        <v>56,0</v>
+        <v>43,4</v>
       </c>
       <c r="F268" t="str">
         <v>98979-8</v>
@@ -7282,7 +7282,7 @@
         <v>w</v>
       </c>
       <c r="H268">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="269">
@@ -7290,7 +7290,7 @@
         <v>9</v>
       </c>
       <c r="B269" s="1">
-        <v>44228.041666666664</v>
+        <v>44713.083333333336</v>
       </c>
       <c r="C269" t="str">
         <v>eGFR</v>
@@ -7299,7 +7299,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E269" t="str">
-        <v>50,0</v>
+        <v>37,9</v>
       </c>
       <c r="F269" t="str">
         <v>98979-8</v>
@@ -7308,7 +7308,7 @@
         <v>w</v>
       </c>
       <c r="H269">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="270">
@@ -7316,7 +7316,7 @@
         <v>9</v>
       </c>
       <c r="B270" s="1">
-        <v>44470.083333333336</v>
+        <v>44958.041666666664</v>
       </c>
       <c r="C270" t="str">
         <v>eGFR</v>
@@ -7325,7 +7325,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E270" t="str">
-        <v>43,4</v>
+        <v>33,0</v>
       </c>
       <c r="F270" t="str">
         <v>98979-8</v>
@@ -7334,7 +7334,7 @@
         <v>w</v>
       </c>
       <c r="H270">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="271">
@@ -7342,7 +7342,7 @@
         <v>9</v>
       </c>
       <c r="B271" s="1">
-        <v>44713.083333333336</v>
+        <v>45200.083333333336</v>
       </c>
       <c r="C271" t="str">
         <v>eGFR</v>
@@ -7351,7 +7351,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E271" t="str">
-        <v>37,9</v>
+        <v>29,2</v>
       </c>
       <c r="F271" t="str">
         <v>98979-8</v>
@@ -7360,7 +7360,7 @@
         <v>w</v>
       </c>
       <c r="H271">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="272">
@@ -7368,7 +7368,7 @@
         <v>9</v>
       </c>
       <c r="B272" s="1">
-        <v>44958.041666666664</v>
+        <v>45444.083333333336</v>
       </c>
       <c r="C272" t="str">
         <v>eGFR</v>
@@ -7377,7 +7377,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E272" t="str">
-        <v>33,0</v>
+        <v>25,7</v>
       </c>
       <c r="F272" t="str">
         <v>98979-8</v>
@@ -7386,7 +7386,7 @@
         <v>w</v>
       </c>
       <c r="H272">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="273">
@@ -7394,7 +7394,7 @@
         <v>9</v>
       </c>
       <c r="B273" s="1">
-        <v>45200.083333333336</v>
+        <v>45689.041666666664</v>
       </c>
       <c r="C273" t="str">
         <v>eGFR</v>
@@ -7403,7 +7403,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E273" t="str">
-        <v>29,2</v>
+        <v>22,6</v>
       </c>
       <c r="F273" t="str">
         <v>98979-8</v>
@@ -7412,15 +7412,15 @@
         <v>w</v>
       </c>
       <c r="H273">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="274">
       <c r="A274">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B274" s="1">
-        <v>45444.083333333336</v>
+        <v>44197.041666666664</v>
       </c>
       <c r="C274" t="str">
         <v>eGFR</v>
@@ -7429,7 +7429,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E274" t="str">
-        <v>25,7</v>
+        <v>59,1</v>
       </c>
       <c r="F274" t="str">
         <v>98979-8</v>
@@ -7438,15 +7438,15 @@
         <v>w</v>
       </c>
       <c r="H274">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="275">
       <c r="A275">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B275" s="1">
-        <v>45689.041666666664</v>
+        <v>44199.041666666664</v>
       </c>
       <c r="C275" t="str">
         <v>eGFR</v>
@@ -7455,7 +7455,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E275" t="str">
-        <v>22,6</v>
+        <v>39,5</v>
       </c>
       <c r="F275" t="str">
         <v>98979-8</v>
@@ -7464,7 +7464,7 @@
         <v>w</v>
       </c>
       <c r="H275">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="276">
@@ -7472,7 +7472,7 @@
         <v>12</v>
       </c>
       <c r="B276" s="1">
-        <v>44197.041666666664</v>
+        <v>44216.041666666664</v>
       </c>
       <c r="C276" t="str">
         <v>eGFR</v>
@@ -7481,7 +7481,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E276" t="str">
-        <v>59,1</v>
+        <v>55,8</v>
       </c>
       <c r="F276" t="str">
         <v>98979-8</v>
@@ -7498,7 +7498,7 @@
         <v>12</v>
       </c>
       <c r="B277" s="1">
-        <v>44199.041666666664</v>
+        <v>44242.041666666664</v>
       </c>
       <c r="C277" t="str">
         <v>eGFR</v>
@@ -7507,7 +7507,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E277" t="str">
-        <v>39,5</v>
+        <v>59,1</v>
       </c>
       <c r="F277" t="str">
         <v>98979-8</v>
@@ -7524,7 +7524,7 @@
         <v>12</v>
       </c>
       <c r="B278" s="1">
-        <v>44216.041666666664</v>
+        <v>44244.041666666664</v>
       </c>
       <c r="C278" t="str">
         <v>eGFR</v>
@@ -7533,7 +7533,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E278" t="str">
-        <v>55,8</v>
+        <v>41,2</v>
       </c>
       <c r="F278" t="str">
         <v>98979-8</v>
@@ -7550,7 +7550,7 @@
         <v>12</v>
       </c>
       <c r="B279" s="1">
-        <v>44242.041666666664</v>
+        <v>44265.041666666664</v>
       </c>
       <c r="C279" t="str">
         <v>eGFR</v>
@@ -7559,7 +7559,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E279" t="str">
-        <v>59,1</v>
+        <v>55,8</v>
       </c>
       <c r="F279" t="str">
         <v>98979-8</v>
@@ -7576,7 +7576,7 @@
         <v>12</v>
       </c>
       <c r="B280" s="1">
-        <v>44244.041666666664</v>
+        <v>44287.083333333336</v>
       </c>
       <c r="C280" t="str">
         <v>eGFR</v>
@@ -7585,7 +7585,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E280" t="str">
-        <v>41,2</v>
+        <v>59,1</v>
       </c>
       <c r="F280" t="str">
         <v>98979-8</v>
@@ -7602,7 +7602,7 @@
         <v>12</v>
       </c>
       <c r="B281" s="1">
-        <v>44265.041666666664</v>
+        <v>44289.083333333336</v>
       </c>
       <c r="C281" t="str">
         <v>eGFR</v>
@@ -7611,7 +7611,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E281" t="str">
-        <v>55,8</v>
+        <v>25,0</v>
       </c>
       <c r="F281" t="str">
         <v>98979-8</v>
@@ -7628,7 +7628,7 @@
         <v>12</v>
       </c>
       <c r="B282" s="1">
-        <v>44287.083333333336</v>
+        <v>44306.083333333336</v>
       </c>
       <c r="C282" t="str">
         <v>eGFR</v>
@@ -7637,7 +7637,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E282" t="str">
-        <v>59,1</v>
+        <v>47,5</v>
       </c>
       <c r="F282" t="str">
         <v>98979-8</v>
@@ -7654,7 +7654,7 @@
         <v>12</v>
       </c>
       <c r="B283" s="1">
-        <v>44289.083333333336</v>
+        <v>44348.083333333336</v>
       </c>
       <c r="C283" t="str">
         <v>eGFR</v>
@@ -7663,7 +7663,7 @@
         <v>ml/min/1,73m²</v>
       </c>
       <c r="E283" t="str">
-        <v>25,0</v>
+        <v>53,9</v>
       </c>
       <c r="F283" t="str">
         <v>98979-8</v>
@@ -7675,61 +7675,9 @@
         <v>74</v>
       </c>
     </row>
-    <row r="284">
-      <c r="A284">
-        <v>12</v>
-      </c>
-      <c r="B284" s="1">
-        <v>44306.083333333336</v>
-      </c>
-      <c r="C284" t="str">
-        <v>eGFR</v>
-      </c>
-      <c r="D284" t="str">
-        <v>ml/min/1,73m²</v>
-      </c>
-      <c r="E284" t="str">
-        <v>47,5</v>
-      </c>
-      <c r="F284" t="str">
-        <v>98979-8</v>
-      </c>
-      <c r="G284" t="str">
-        <v>w</v>
-      </c>
-      <c r="H284">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285">
-        <v>12</v>
-      </c>
-      <c r="B285" s="1">
-        <v>44348.083333333336</v>
-      </c>
-      <c r="C285" t="str">
-        <v>eGFR</v>
-      </c>
-      <c r="D285" t="str">
-        <v>ml/min/1,73m²</v>
-      </c>
-      <c r="E285" t="str">
-        <v>53,9</v>
-      </c>
-      <c r="F285" t="str">
-        <v>98979-8</v>
-      </c>
-      <c r="G285" t="str">
-        <v>w</v>
-      </c>
-      <c r="H285">
-        <v>74</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H285"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H283"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Address review: qualifying group sizes, demo margin, separators
- Group sizes count patients the validation accepts (qualifyingMixedModelPatients
  in validation.ts); the 'no group can be fitted' sentence appears only when
  every group fails for lack of such patients, otherwise the per-unit reasons
  stay. Sizes read 'A: 12' so numeric group values stay unambiguous.
- Two more cohort-A demo patients (27, 28) keep cohort A above the minimum under
  CKD progression; the demo test checks cohort and sex groupings under both
  presets.
- Method reference describes the group-size line and 'Fit whole cohort only'.
- Endpoint tooltips use one sentence per item, point tooltips put exclusion
  reasons in brackets, chart titles read 'eGFR by calendar date', eyebrow
  'Patients and trajectories'; changelog states which phrases changed.
- Dated smoke checklist entry.
</commit_message>
<xml_diff>
--- a/public/test_labs.xlsx
+++ b/public/test_labs.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H475"/>
+  <dimension ref="A1:H507"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12667,9 +12667,841 @@
         <v>62</v>
       </c>
     </row>
+    <row r="476">
+      <c r="A476">
+        <v>27</v>
+      </c>
+      <c r="B476" s="1">
+        <v>44659.083333333336</v>
+      </c>
+      <c r="C476" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D476" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E476" t="str">
+        <v>0,91</v>
+      </c>
+      <c r="F476" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G476" t="str">
+        <v>w</v>
+      </c>
+      <c r="H476">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477">
+        <v>27</v>
+      </c>
+      <c r="B477" s="1">
+        <v>44659.083333333336</v>
+      </c>
+      <c r="C477" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D477" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E477" t="str">
+        <v>77,3</v>
+      </c>
+      <c r="F477" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G477" t="str">
+        <v>w</v>
+      </c>
+      <c r="H477">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478">
+        <v>27</v>
+      </c>
+      <c r="B478" s="1">
+        <v>44850.083333333336</v>
+      </c>
+      <c r="C478" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D478" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E478" t="str">
+        <v>0,89</v>
+      </c>
+      <c r="F478" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G478" t="str">
+        <v>w</v>
+      </c>
+      <c r="H478">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479">
+        <v>27</v>
+      </c>
+      <c r="B479" s="1">
+        <v>44850.083333333336</v>
+      </c>
+      <c r="C479" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D479" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E479" t="str">
+        <v>79,4</v>
+      </c>
+      <c r="F479" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G479" t="str">
+        <v>w</v>
+      </c>
+      <c r="H479">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480">
+        <v>27</v>
+      </c>
+      <c r="B480" s="1">
+        <v>45035.083333333336</v>
+      </c>
+      <c r="C480" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D480" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E480" t="str">
+        <v>0,96</v>
+      </c>
+      <c r="F480" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G480" t="str">
+        <v>w</v>
+      </c>
+      <c r="H480">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481">
+        <v>27</v>
+      </c>
+      <c r="B481" s="1">
+        <v>45035.083333333336</v>
+      </c>
+      <c r="C481" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D481" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E481" t="str">
+        <v>72,1</v>
+      </c>
+      <c r="F481" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G481" t="str">
+        <v>w</v>
+      </c>
+      <c r="H481">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482">
+        <v>27</v>
+      </c>
+      <c r="B482" s="1">
+        <v>45220.083333333336</v>
+      </c>
+      <c r="C482" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D482" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E482" t="str">
+        <v>0,95</v>
+      </c>
+      <c r="F482" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G482" t="str">
+        <v>w</v>
+      </c>
+      <c r="H482">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483">
+        <v>27</v>
+      </c>
+      <c r="B483" s="1">
+        <v>45220.083333333336</v>
+      </c>
+      <c r="C483" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D483" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E483" t="str">
+        <v>73,0</v>
+      </c>
+      <c r="F483" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G483" t="str">
+        <v>w</v>
+      </c>
+      <c r="H483">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484">
+        <v>27</v>
+      </c>
+      <c r="B484" s="1">
+        <v>45389.083333333336</v>
+      </c>
+      <c r="C484" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D484" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E484" t="str">
+        <v>0,99</v>
+      </c>
+      <c r="F484" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G484" t="str">
+        <v>w</v>
+      </c>
+      <c r="H484">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485">
+        <v>27</v>
+      </c>
+      <c r="B485" s="1">
+        <v>45389.083333333336</v>
+      </c>
+      <c r="C485" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D485" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E485" t="str">
+        <v>69,0</v>
+      </c>
+      <c r="F485" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G485" t="str">
+        <v>w</v>
+      </c>
+      <c r="H485">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486">
+        <v>27</v>
+      </c>
+      <c r="B486" s="1">
+        <v>45582.083333333336</v>
+      </c>
+      <c r="C486" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D486" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E486" t="str">
+        <v>1,06</v>
+      </c>
+      <c r="F486" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G486" t="str">
+        <v>w</v>
+      </c>
+      <c r="H486">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487">
+        <v>27</v>
+      </c>
+      <c r="B487" s="1">
+        <v>45582.083333333336</v>
+      </c>
+      <c r="C487" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D487" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E487" t="str">
+        <v>63,6</v>
+      </c>
+      <c r="F487" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G487" t="str">
+        <v>w</v>
+      </c>
+      <c r="H487">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488">
+        <v>27</v>
+      </c>
+      <c r="B488" s="1">
+        <v>45762.083333333336</v>
+      </c>
+      <c r="C488" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D488" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E488" t="str">
+        <v>1,06</v>
+      </c>
+      <c r="F488" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G488" t="str">
+        <v>w</v>
+      </c>
+      <c r="H488">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489">
+        <v>27</v>
+      </c>
+      <c r="B489" s="1">
+        <v>45762.083333333336</v>
+      </c>
+      <c r="C489" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D489" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E489" t="str">
+        <v>63,2</v>
+      </c>
+      <c r="F489" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G489" t="str">
+        <v>w</v>
+      </c>
+      <c r="H489">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490">
+        <v>27</v>
+      </c>
+      <c r="B490" s="1">
+        <v>45939.083333333336</v>
+      </c>
+      <c r="C490" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D490" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E490" t="str">
+        <v>1,16</v>
+      </c>
+      <c r="F490" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G490" t="str">
+        <v>w</v>
+      </c>
+      <c r="H490">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491">
+        <v>27</v>
+      </c>
+      <c r="B491" s="1">
+        <v>45939.083333333336</v>
+      </c>
+      <c r="C491" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D491" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E491" t="str">
+        <v>56,7</v>
+      </c>
+      <c r="F491" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G491" t="str">
+        <v>w</v>
+      </c>
+      <c r="H491">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492">
+        <v>28</v>
+      </c>
+      <c r="B492" s="1">
+        <v>43885.041666666664</v>
+      </c>
+      <c r="C492" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D492" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E492" t="str">
+        <v>1,14</v>
+      </c>
+      <c r="F492" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G492" t="str">
+        <v>m</v>
+      </c>
+      <c r="H492">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493">
+        <v>28</v>
+      </c>
+      <c r="B493" s="1">
+        <v>43885.041666666664</v>
+      </c>
+      <c r="C493" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D493" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E493" t="str">
+        <v>75,5</v>
+      </c>
+      <c r="F493" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G493" t="str">
+        <v>m</v>
+      </c>
+      <c r="H493">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494">
+        <v>28</v>
+      </c>
+      <c r="B494" s="1">
+        <v>44058.083333333336</v>
+      </c>
+      <c r="C494" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D494" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E494" t="str">
+        <v>1,17</v>
+      </c>
+      <c r="F494" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G494" t="str">
+        <v>m</v>
+      </c>
+      <c r="H494">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495">
+        <v>28</v>
+      </c>
+      <c r="B495" s="1">
+        <v>44058.083333333336</v>
+      </c>
+      <c r="C495" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D495" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E495" t="str">
+        <v>73,2</v>
+      </c>
+      <c r="F495" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G495" t="str">
+        <v>m</v>
+      </c>
+      <c r="H495">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496">
+        <v>28</v>
+      </c>
+      <c r="B496" s="1">
+        <v>44242.041666666664</v>
+      </c>
+      <c r="C496" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D496" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E496" t="str">
+        <v>1,13</v>
+      </c>
+      <c r="F496" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G496" t="str">
+        <v>m</v>
+      </c>
+      <c r="H496">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497">
+        <v>28</v>
+      </c>
+      <c r="B497" s="1">
+        <v>44242.041666666664</v>
+      </c>
+      <c r="C497" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D497" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E497" t="str">
+        <v>75,8</v>
+      </c>
+      <c r="F497" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G497" t="str">
+        <v>m</v>
+      </c>
+      <c r="H497">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498">
+        <v>28</v>
+      </c>
+      <c r="B498" s="1">
+        <v>44423.083333333336</v>
+      </c>
+      <c r="C498" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D498" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E498" t="str">
+        <v>1,17</v>
+      </c>
+      <c r="F498" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G498" t="str">
+        <v>m</v>
+      </c>
+      <c r="H498">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499">
+        <v>28</v>
+      </c>
+      <c r="B499" s="1">
+        <v>44423.083333333336</v>
+      </c>
+      <c r="C499" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D499" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E499" t="str">
+        <v>72,7</v>
+      </c>
+      <c r="F499" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G499" t="str">
+        <v>m</v>
+      </c>
+      <c r="H499">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500">
+        <v>28</v>
+      </c>
+      <c r="B500" s="1">
+        <v>44602.041666666664</v>
+      </c>
+      <c r="C500" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D500" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E500" t="str">
+        <v>1,16</v>
+      </c>
+      <c r="F500" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G500" t="str">
+        <v>m</v>
+      </c>
+      <c r="H500">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501">
+        <v>28</v>
+      </c>
+      <c r="B501" s="1">
+        <v>44602.041666666664</v>
+      </c>
+      <c r="C501" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D501" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E501" t="str">
+        <v>73,0</v>
+      </c>
+      <c r="F501" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G501" t="str">
+        <v>m</v>
+      </c>
+      <c r="H501">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502">
+        <v>28</v>
+      </c>
+      <c r="B502" s="1">
+        <v>44788.083333333336</v>
+      </c>
+      <c r="C502" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D502" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E502" t="str">
+        <v>1,23</v>
+      </c>
+      <c r="F502" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G502" t="str">
+        <v>m</v>
+      </c>
+      <c r="H502">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503">
+        <v>28</v>
+      </c>
+      <c r="B503" s="1">
+        <v>44788.083333333336</v>
+      </c>
+      <c r="C503" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D503" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E503" t="str">
+        <v>68,1</v>
+      </c>
+      <c r="F503" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G503" t="str">
+        <v>m</v>
+      </c>
+      <c r="H503">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504">
+        <v>28</v>
+      </c>
+      <c r="B504" s="1">
+        <v>44972.041666666664</v>
+      </c>
+      <c r="C504" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D504" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E504" t="str">
+        <v>1,22</v>
+      </c>
+      <c r="F504" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G504" t="str">
+        <v>m</v>
+      </c>
+      <c r="H504">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505">
+        <v>28</v>
+      </c>
+      <c r="B505" s="1">
+        <v>44972.041666666664</v>
+      </c>
+      <c r="C505" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D505" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E505" t="str">
+        <v>68,3</v>
+      </c>
+      <c r="F505" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G505" t="str">
+        <v>m</v>
+      </c>
+      <c r="H505">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506">
+        <v>28</v>
+      </c>
+      <c r="B506" s="1">
+        <v>45151.083333333336</v>
+      </c>
+      <c r="C506" t="str">
+        <v>Kreatinin</v>
+      </c>
+      <c r="D506" t="str">
+        <v>mg/dl</v>
+      </c>
+      <c r="E506" t="str">
+        <v>1,32</v>
+      </c>
+      <c r="F506" t="str">
+        <v>2160-0</v>
+      </c>
+      <c r="G506" t="str">
+        <v>m</v>
+      </c>
+      <c r="H506">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507">
+        <v>28</v>
+      </c>
+      <c r="B507" s="1">
+        <v>45151.083333333336</v>
+      </c>
+      <c r="C507" t="str">
+        <v>eGFR</v>
+      </c>
+      <c r="D507" t="str">
+        <v>ml/min/1,73m²</v>
+      </c>
+      <c r="E507" t="str">
+        <v>62,1</v>
+      </c>
+      <c r="F507" t="str">
+        <v>98979-8</v>
+      </c>
+      <c r="G507" t="str">
+        <v>m</v>
+      </c>
+      <c r="H507">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H475"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H507"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12855,7 +13687,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13201,9 +14033,37 @@
         <v>B</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26">
+        <v>27</v>
+      </c>
+      <c r="B26" t="str">
+        <v>UMOD</v>
+      </c>
+      <c r="C26" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D26" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>28</v>
+      </c>
+      <c r="B27" t="str">
+        <v>UMOD</v>
+      </c>
+      <c r="C27" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D27" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>